<commit_message>
Finalize working specification PDF and fix Z594470 name
Independent re-read of all 14 scanned pages found one transcription
error: the Russian name of Z594470 reads «КЛЕШЕ (ПАТРОН) КАЛИБРОВОЧНЫЙ»
(with Ш), not «КЛЕЩЕ». Corrected in the Excel workbook and the PDF;
all other 40 lines and printed totals confirmed. PDF layout tightened
to 4 pages.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0178Q7WcpmJCR7PcxckJf1X5
</commit_message>
<xml_diff>
--- a/specification_UZ95-039-045-2026.xlsx
+++ b/specification_UZ95-039-045-2026.xlsx
@@ -84,7 +84,7 @@
     <t xml:space="preserve">9015 90 — части и принадлежности; товар — готовый прибор (зам. 7)</t>
   </si>
   <si>
-    <t xml:space="preserve">Неясное слово «КЛЕЩЕ» (зам. 9); код 9015 90 — части и принадлежности (зам. 7)</t>
+    <t xml:space="preserve">Неясное слово «КЛЕШЕ» (зам. 9); код 9015 90 — части и принадлежности (зам. 7)</t>
   </si>
   <si>
     <t xml:space="preserve">Опечатка: верно «ЭЛЕКТРОПНЕВМАТИЧЕСКИЙ» — перенесено как в оригинале (зам. 8)</t>
@@ -366,7 +366,7 @@
     <t xml:space="preserve">PATRON REPARADO/CALIBRADO</t>
   </si>
   <si>
-    <t xml:space="preserve">КЛЕЩЕ (ПАТРОН) КАЛИБРОВОЧНЫЙ</t>
+    <t xml:space="preserve">КЛЕШЕ (ПАТРОН) КАЛИБРОВОЧНЫЙ</t>
   </si>
   <si>
     <t xml:space="preserve">UZ95-043-2026</t>
@@ -810,7 +810,7 @@
     <t xml:space="preserve">Z10063008, Z594470</t>
   </si>
   <si>
-    <t xml:space="preserve">Код 9015900000 — субпозиция 9015 90 «части и принадлежности». «ЦИФРОВОЙ ИНКЛИНОМЕТР» — законченный прибор, а не часть (возможно, 9015 80). Назначение Z594470 «КЛЕЩЕ (ПАТРОН) КАЛИБРОВОЧНЫЙ» (исп. PATRON — эталон/шаблон) из документов неясно.</t>
+    <t xml:space="preserve">Код 9015900000 — субпозиция 9015 90 «части и принадлежности». «ЦИФРОВОЙ ИНКЛИНОМЕТР» — законченный прибор, а не часть (возможно, 9015 80). Назначение Z594470 «КЛЕШЕ (ПАТРОН) КАЛИБРОВОЧНЫЙ» (исп. PATRON — эталон/шаблон) из документов неясно.</t>
   </si>
   <si>
     <t xml:space="preserve">Коды перенесены как в документе.</t>
@@ -831,13 +831,13 @@
     <t xml:space="preserve">Неясное наименование</t>
   </si>
   <si>
-    <t xml:space="preserve">«КЛЕЩЕ (ПАТРОН) КАЛИБРОВОЧНЫЙ» — «КЛЕЩЕ» не является корректной словоформой (возможно, имелось в виду «КЛЕЩИ»). Исп.: PATRON REPARADO/CALIBRADO — эталон (шаблон) отремонтированный/откалиброванный.</t>
+    <t xml:space="preserve">«КЛЕШЕ (ПАТРОН) КАЛИБРОВОЧНЫЙ» — слова «КЛЕШЕ» в русском языке нет. Возможно, имелось в виду «КЛИШЕ» (шаблон), что согласуется с исп. описанием, но это предположение. Исп.: PATRON REPARADO/CALIBRADO — эталон (шаблон) отремонтированный/откалиброванный.</t>
   </si>
   <si>
     <t xml:space="preserve">Перенесено как в оригинале; уточнить у отправителя.</t>
   </si>
   <si>
-    <t xml:space="preserve">Высокая — в части факта; что имелось в виду, я не знаю</t>
+    <t xml:space="preserve">Высокая — написание подтверждено повторной независимой проверкой скана; версия «КЛИШЕ» — предположение</t>
   </si>
   <si>
     <t xml:space="preserve">Расчёт (не из документа)</t>
@@ -2190,7 +2190,7 @@
       </c>
       <c r="D18" s="6" t="str">
         <f aca="false">'Исходные данные'!K18</f>
-        <v>КЛЕЩЕ (ПАТРОН) КАЛИБРОВОЧНЫЙ</v>
+        <v>КЛЕШЕ (ПАТРОН) КАЛИБРОВОЧНЫЙ</v>
       </c>
       <c r="E18" s="5" t="str">
         <f aca="false">'Исходные данные'!M18</f>

</xml_diff>